<commit_message>
feat(Step 17-D Phase 2-C): 알림 안전 wrapper + auth_failure 배너 + dismiss API
- safe_send_alert: SMTP 실패해도 stderr fallback + DB 누적
- /api/notifications/auth-failures: 24h 내 인증 실패 알림 조회
- /api/notifications/dismiss: 알림 dismiss API
- _refresh_session_if_stale failed 시 auth_failure 알림 발송
- 대시보드 상단 배너: 자동 polling (5분), dismiss 버튼

회귀 테스트: 모두 PASS
</commit_message>
<xml_diff>
--- a/kream_bulk_bid.xlsx
+++ b/kream_bulk_bid.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,17 +510,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>299955</t>
+          <t>X2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IX7694</t>
+          <t>JE3208</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Adidas Always Original Denim Shoulder Bag Black</t>
+          <t>bag</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>76000</v>
+        <v>100000</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
@@ -540,26 +540,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>125755</t>
+          <t>X3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IC8349</t>
+          <t>JQ4110</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Adidas Always Original Shoulder Bag Black</t>
+          <t>shoes</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ONE SIZE</t>
+          <t>230</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>119000</v>
+        <v>100000</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -570,17 +570,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>490300</t>
+          <t>X5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>KA9271</t>
+          <t>JE3209</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Adidas Originals Cloud Shoulder Bag Crinkle Version Large Size Black</t>
+          <t>bag2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -589,343 +589,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>77000</v>
+        <v>100000</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>490299</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>KA9266</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Adidas Crinkle Version Cloud Shoulder Bag Small Black</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>76000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>401633</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>JP0145</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Adidas Originals Cloud Shoulder Bag Large Black</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>85000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>307489</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>JP0146</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Adidas Originals Cloud Shoulder Bag XLarge Black</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>96000</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>125755</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>IC8349</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Adidas Always Original Shoulder Bag Black</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>125000</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>299955</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>IX7694</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Adidas Always Original Denim Shoulder Bag Black</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>78000</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>125755</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>IC8349</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Adidas Always Original Shoulder Bag Black</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>122000</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>299955</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>IX7694</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Adidas Always Original Denim Shoulder Bag Black</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>79000</v>
-      </c>
-      <c r="F13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>490300</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>KA9271</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Adidas Originals Cloud Shoulder Bag Crinkle Version Large Size Black</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>75000</v>
-      </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>490299</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>KA9266</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Adidas Crinkle Version Cloud Shoulder Bag Small Black</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>77000</v>
-      </c>
-      <c r="F15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>307489</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>JP0146</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Adidas Originals Cloud Shoulder Bag XLarge Black</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>99000</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>401633</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>JP0145</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Adidas Originals Cloud Shoulder Bag Large Black</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>ONE SIZE</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>84000</v>
-      </c>
-      <c r="F17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>